<commit_message>
Mise à jour automatique des Bestsellers (Onglets)
</commit_message>
<xml_diff>
--- a/historique_bestsellers.xlsx
+++ b/historique_bestsellers.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D101"/>
+  <dimension ref="A1:D201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2646,6 +2646,2206 @@
         </is>
       </c>
       <c r="D101" t="inlineStr">
+        <is>
+          <t>€10.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>#1</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>B0CNVTCK51</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>€9.88</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>#2</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>B0CNVTCK51</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>€9.88</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>#3</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>B0BPNT6XYY</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>€9.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>#4</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>B0BPNT6XYY</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>€9.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>#5</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>B0F93BDHHF</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>€22.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>#6</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>B0F93BDHHF</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>€22.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>#7</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>B0DJS84VNY</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>€7.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>#8</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>B0DJS84VNY</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>€7.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>#9</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>B0DWXHV7L5</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>€7.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>#10</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>B0DWXHV7L5</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>€7.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>#11</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>B0F6MRMCCQ</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>€9.58</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>#12</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>B0F6MRMCCQ</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>€9.58</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>#13</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>B0FXFX6W31</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>€9.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>#14</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>B0FXFX6W31</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>€9.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>#15</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>B0GHNJ6ZY3</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>€9.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>#16</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>B0GHNJ6ZY3</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>€9.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>#17</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>B0DSZLRYTB</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>€11.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>#18</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>B0DSZLRYTB</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>€11.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>#19</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>B0DLKLY2RS</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>€21.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>#20</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>B0DLKLY2RS</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>€21.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>#21</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>B0GCHZ4RP5</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>€21.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>#22</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>B0GCHZ4RP5</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>€21.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>#23</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>B0DJTDNSQN</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>€7.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>#24</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>B0DJTDNSQN</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>€7.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>#25</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>B0C2CM7QWR</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>€14.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>#26</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>B0C2CM7QWR</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>€14.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>#27</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>B0DM4WJ7XH</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>€6.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>#28</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>B0DM4WJ7XH</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>€6.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>#29</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>B0DSW4V65Z</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>€7.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>#30</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>B0DSW4V65Z</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>€7.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>#31</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>B0DSZXH6BG</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>€9.58</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>#32</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>B0DSZXH6BG</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>€9.58</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>#33</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>B0DWSTJ4HS</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>€17.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>#34</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>B0DWSTJ4HS</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>€17.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>#35</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>B0DK8SYX8F</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>€9.44</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>#36</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>B0DK8SYX8F</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>€9.44</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>#37</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>B0DK9528FW</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>€9.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>#38</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>B0DK9528FW</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>€9.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>#39</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>B0CFV96666</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>€10.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>#40</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>B0CFV96666</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>€10.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>#41</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>B0F9YKRBCJ</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>€8.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>#42</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>B0F9YKRBCJ</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>€8.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>#43</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>B0D7YT3ZMX</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>€8.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>#44</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>B0D7YT3ZMX</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>€8.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>#45</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>B0CYGJ2RNV</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>€9.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>#46</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>B0CYGJ2RNV</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>€9.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>#47</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>B0F2MV5NGP</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>€21.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>#48</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>B0F2MV5NGP</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>€21.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>#49</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>B0FXG8CR1V</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>€9.58</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>#50</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>B0FXG8CR1V</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>€9.58</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>#51</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>B0BTH76GS7</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>€10.49</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>#52</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>B0BTH76GS7</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>€10.49</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>#53</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>B0FFYWVP45</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>€11.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>#54</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>B0FFYWVP45</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>€11.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>#55</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>B0G6C44RPY</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>€10.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>#56</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>B0G6C44RPY</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>€10.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>#57</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>B0F6LP1M79</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>€11.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>#58</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>B0F6LP1M79</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>€11.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>#59</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>B0GDJSFDL4</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>€6.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>#60</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>B0GDJSFDL4</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>€6.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>#61</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>B0F6CNSRNC</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>€6.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>#62</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>B0F6CNSRNC</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>€6.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>#63</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>B0FFSF5NHR</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>€10.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>#64</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>B0FFSF5NHR</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>€10.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>#65</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>B0FXX82RGG</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>€17.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>#66</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>B0FXX82RGG</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>€17.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>#67</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>B0GJN22NJV</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>€7.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>#68</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>B0GJN22NJV</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>€7.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>#69</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>B0FVL3BV29</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>€21.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>#70</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>B0FVL3BV29</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>€21.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>#71</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>B0DFPRVGN7</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>€5.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>#72</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>B0DFPRVGN7</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>€5.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>#73</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>B0FDKND69M</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>€13.48</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>#74</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>B0FDKND69M</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>€13.48</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>#75</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>B0DM5YLYHB</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>€6.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>#76</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>B0DM5YLYHB</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>€6.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>#77</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>B0D5JRJCVX</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>€12.74</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>#78</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>B0D5JRJCVX</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>€12.74</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>#79</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>B0GF6SBD6J</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>€6.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>#80</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>B0GF6SBD6J</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>€6.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>#81</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>B0G3WZMGZJ</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>€6.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>#82</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>B0G3WZMGZJ</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>€6.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>#83</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>B0DDSPNKNT</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>€12.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>#84</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>B0DDSPNKNT</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>€12.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>#85</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>B0FJY96R5S</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>€6.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>#86</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>B0FJY96R5S</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>€6.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>#87</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>B0DJTD19WX</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>€7.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>#88</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>B0DJTD19WX</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>€7.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>#89</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>B0FPF2PBNM</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>€7.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>#90</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>B0FPF2PBNM</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>€7.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>#91</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>B0D8KHVX7S</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>€10.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>#92</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>B0D8KHVX7S</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>€10.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>#93</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>B0CCND87VQ</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>€8.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>#94</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>B0CCND87VQ</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>€8.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>#95</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>B0F2GHWNK3</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>€6.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>#96</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>B0F2GHWNK3</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>€6.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>#97</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>B0DXZZKPQ3</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>€7.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>#98</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>B0DXZZKPQ3</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>€7.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>#99</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>B0F5B537XQ</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>€10.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>#100</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>B0F5B537XQ</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
         <is>
           <t>€10.99</t>
         </is>

</xml_diff>

<commit_message>
Mise à jour automatique des Bestsellers et Fiches Produits
</commit_message>
<xml_diff>
--- a/historique_bestsellers.xlsx
+++ b/historique_bestsellers.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D201"/>
+  <dimension ref="A1:D301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4846,6 +4846,2206 @@
         </is>
       </c>
       <c r="D201" t="inlineStr">
+        <is>
+          <t>€10.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>#1</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>B0CNVTCK51</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>€9.88</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>#2</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>B0CNVTCK51</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>€9.88</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>#3</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>B0BPNT6XYY</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>€9.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>#4</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>B0BPNT6XYY</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>€9.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>#5</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>B0F93BDHHF</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>€22.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>#6</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>B0F93BDHHF</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>€22.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>#7</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>B0DJS84VNY</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>€7.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>#8</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>B0DJS84VNY</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>€7.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>#9</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>B0DWXHV7L5</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>€7.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>#10</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>B0DWXHV7L5</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>€7.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>#11</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>B0F6MRMCCQ</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>€9.58</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>#12</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>B0F6MRMCCQ</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>€9.58</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>#13</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>B0FXFX6W31</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>€9.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>#14</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>B0FXFX6W31</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>€9.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>#15</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>B0GHNJ6ZY3</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>€9.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>#16</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>B0GHNJ6ZY3</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>€9.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>#17</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>B0DSZLRYTB</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>€11.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>#18</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>B0DSZLRYTB</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>€11.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>#19</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>B0DLKLY2RS</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>€21.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>#20</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>B0DLKLY2RS</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>€21.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>#21</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>B0GCHZ4RP5</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>€21.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>#22</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>B0GCHZ4RP5</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>€21.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>#23</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>B0DJTDNSQN</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>€7.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>#24</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>B0DJTDNSQN</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>€7.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>#25</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>B0C2CM7QWR</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>€14.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>#26</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>B0C2CM7QWR</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>€14.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>#27</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>B0DM4WJ7XH</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>€6.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>#28</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>B0DM4WJ7XH</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>€6.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>#29</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>B0DSW4V65Z</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>€7.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>#30</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>B0DSW4V65Z</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>€7.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>#31</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>B0DSZXH6BG</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>€9.58</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>#32</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>B0DSZXH6BG</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>€9.58</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>#33</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>B0DWSTJ4HS</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>€17.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>#34</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>B0DWSTJ4HS</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>€17.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>#35</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>B0DK8SYX8F</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>€9.44</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>#36</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>B0DK8SYX8F</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>€9.44</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>#37</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>B0DK9528FW</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>€9.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>#38</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>B0DK9528FW</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>€9.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>#39</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>B0CFV96666</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>€10.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>#40</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>B0CFV96666</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>€10.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>#41</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>B0F9YKRBCJ</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>€8.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>#42</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>B0F9YKRBCJ</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>€8.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>#43</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>B0D7YT3ZMX</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>€8.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>#44</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>B0D7YT3ZMX</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>€8.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>#45</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>B0CYGJ2RNV</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>€9.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>#46</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>B0CYGJ2RNV</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>€9.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>#47</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>B0F2MV5NGP</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>€21.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>#48</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>B0F2MV5NGP</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>€21.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>#49</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>B0FXG8CR1V</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>€9.58</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>#50</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>B0FXG8CR1V</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>€9.58</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>#51</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>B0BTH76GS7</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>€10.49</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>#52</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>B0BTH76GS7</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>€10.49</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>#53</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>B0FFYWVP45</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>€11.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>#54</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>B0FFYWVP45</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>€11.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>#55</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>B0G6C44RPY</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>€10.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>#56</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>B0G6C44RPY</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>€10.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>#57</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>B0F6LP1M79</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>€11.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>#58</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>B0F6LP1M79</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>€11.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>#59</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>B0GDJSFDL4</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>€6.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>#60</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>B0GDJSFDL4</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>€6.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>#61</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>B0F6CNSRNC</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>€6.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>#62</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>B0F6CNSRNC</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>€6.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>#63</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>B0FFSF5NHR</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>€10.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>#64</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>B0FFSF5NHR</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>€10.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>#65</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>B0FXX82RGG</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>€17.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>#66</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>B0FXX82RGG</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>€17.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>#67</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>B0GJN22NJV</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>€7.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>#68</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>B0GJN22NJV</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>€7.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>#69</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>B0FVL3BV29</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>€21.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>#70</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>B0FVL3BV29</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>€21.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>#71</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>B0DFPRVGN7</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>€5.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>#72</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>B0DFPRVGN7</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>€5.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>#73</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>B0FDKND69M</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>€13.48</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>#74</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>B0FDKND69M</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>€13.48</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>#75</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>B0DM5YLYHB</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>€6.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>#76</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>B0DM5YLYHB</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>€6.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>#77</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>B0D5JRJCVX</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>€12.74</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>#78</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>B0D5JRJCVX</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>€12.74</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>#79</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>B0GF6SBD6J</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>€6.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>#80</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>B0GF6SBD6J</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>€6.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>#81</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>B0G3WZMGZJ</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>€6.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>#82</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>B0G3WZMGZJ</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>€6.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>#83</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>B0DDSPNKNT</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>€12.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>#84</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>B0DDSPNKNT</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>€12.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>#85</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>B0FJY96R5S</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>€6.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>#86</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>B0FJY96R5S</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>€6.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>#87</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>B0DJTD19WX</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>€7.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>#88</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>B0DJTD19WX</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>€7.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>#89</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>B0FPF2PBNM</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>€7.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>#90</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>B0FPF2PBNM</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>€7.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>#91</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>B0D8KHVX7S</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>€10.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>#92</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>B0D8KHVX7S</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>€10.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>#93</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>B0CCND87VQ</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>€8.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>#94</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>B0CCND87VQ</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>€8.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>#95</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>B0F2GHWNK3</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>€6.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>#96</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>B0F2GHWNK3</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>€6.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>#97</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>B0DXZZKPQ3</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>€7.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>#98</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>B0DXZZKPQ3</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>€7.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>#99</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>B0F5B537XQ</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>€10.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>#100</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>B0F5B537XQ</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
         <is>
           <t>€10.99</t>
         </is>
@@ -4862,7 +7062,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:P51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4896,6 +7096,56 @@
           <t>Date_Detection</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Titre_Complet</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Nb_Avis</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Bullet_Points</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Nombre_Images</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Caracteristiques</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>BSR_Categories</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Declinaisons</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Nb_Declinaisons</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Date_Analyse</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -4910,12 +7160,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>À collecter en Phase 2</t>
+          <t>Inconnu</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>À collecter en Phase 2</t>
+          <t>Aucune description textuelle</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -4924,6 +7174,52 @@
         </is>
       </c>
       <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Inconnu</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Pas de note</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Aucun</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Aucune caractéristique trouvée</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Inconnu</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Aucune déclinaison</t>
+        </is>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
@@ -4942,12 +7238,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>À collecter en Phase 2</t>
+          <t>Inconnu</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>À collecter en Phase 2</t>
+          <t>Aucune description textuelle</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -4956,6 +7252,52 @@
         </is>
       </c>
       <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Inconnu</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Pas de note</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Aucun</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Aucune caractéristique trouvée</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Inconnu</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Aucune déclinaison</t>
+        </is>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
@@ -4974,12 +7316,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>À collecter en Phase 2</t>
+          <t>Inconnu</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>À collecter en Phase 2</t>
+          <t>Aucune description textuelle</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -4988,6 +7330,52 @@
         </is>
       </c>
       <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Inconnu</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Pas de note</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Aucun</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Aucune caractéristique trouvée</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Inconnu</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Aucune déclinaison</t>
+        </is>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
@@ -5006,12 +7394,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>À collecter en Phase 2</t>
+          <t>Inconnu</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>À collecter en Phase 2</t>
+          <t>Aucune description textuelle</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -5020,6 +7408,52 @@
         </is>
       </c>
       <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Inconnu</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Pas de note</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Aucun</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Aucune caractéristique trouvée</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Inconnu</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Aucune déclinaison</t>
+        </is>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
@@ -5038,12 +7472,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>À collecter en Phase 2</t>
+          <t>Inconnu</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>À collecter en Phase 2</t>
+          <t>Aucune description textuelle</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -5052,6 +7486,52 @@
         </is>
       </c>
       <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Inconnu</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Pas de note</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Aucun</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Aucune caractéristique trouvée</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Inconnu</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Aucune déclinaison</t>
+        </is>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
@@ -5070,12 +7550,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>À collecter en Phase 2</t>
+          <t>Inconnu</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>À collecter en Phase 2</t>
+          <t>Aucune description textuelle</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -5084,6 +7564,52 @@
         </is>
       </c>
       <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Inconnu</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Pas de note</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Aucun</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Aucune caractéristique trouvée</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Inconnu</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Aucune déclinaison</t>
+        </is>
+      </c>
+      <c r="O7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
@@ -5102,12 +7628,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>À collecter en Phase 2</t>
+          <t>Visit the HWeggo Store</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>À collecter en Phase 2</t>
+          <t>Aucune description textuelle</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -5116,6 +7642,52 @@
         </is>
       </c>
       <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>[2 in 1] Waterproof Case for Apple Watch Series Ultra 3/Ultra 2/Ultra 49mm Accessories, 360° Front and Back, iWatch PC Screen Protector with Tempered Glass for Women and Men, 49mm Black</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>4.3 out of 5 stars</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>(2,040)</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>【COMPATIBILITY】Tensea iWatch screen protector with back cover is designed to fit Apple Watch Ultra 3 49mm, Apple Watch Ultra 2 49mm and Apple Watch Ultra 49mm. The bumper cover built into the screen protector provides a perfect fit. | 【Daily Water Resistance】 Apple Watch Ultra 3/Ultra 2/Ultra 49mm has a built-in seal that effectively prevents water from entering the screen. Its exceptional water resistance for everyday use makes it possible to use it with confidence during activities such as showering, hand washing, sweating or showering. [Note: Not suitable for deep water environments such as diving or swimming.] | 【360°Protection】This protective case, compatible with the surface of iWatch Ultra 3/Ultra 2/Ultra 49mm, provides full protection to the front and back of your watch, effectively resisting dust, dirt, scratches and damage. The 9H tempered glass screen protector preserves touch sensitivity, while the sweat-resistant case design allows for easy installation without having to remove the band. | 【Upgraded Materials】 Scratch-resistant and impact-resistant tempered glass has a hardness of 9H. Shock absorbing polycarbonate provides superior rigidity, improved resilience and better protection compared to conventional TPU. Glass construction prevents fogging caused by temperature fluctuations. | 【Easy Installation】The product page includes installation video and the package contains installation instructions. A removal tool is provided to allow the watch case to be removed without damaging it.</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>7</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Aucune caractéristique trouvée</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Inconnu</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Aucune déclinaison</t>
+        </is>
+      </c>
+      <c r="O8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
@@ -5134,20 +7706,62 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>À collecter en Phase 2</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>À collecter en Phase 2</t>
-        </is>
-      </c>
+          <t>Brand: TUTUO</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>À collecter en Phase 2</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>TUTUO For Garmin Forerunner 165/165 Music Case, [2 Pieces] Full Coverage Protective Case with Screen Protector, Anti-Scratch Shockproof TPU Case – Transparent+Black</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>4.4 out of 5 stars</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>(61)</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Compatible Model: Compatible with Garmin Forerunner 165 / 165 Music. Precise design will fit your watch perfectly. (Note: Please check your watch model number before purchasing) | Full protection: The protective case for Garmin Forerunner 165 / 165 Music offers full screen protection from four sides to the corners. Slightly higher edges protect the surface of your watch and protect it from scratches, bumps and accidental drops. | Effective protective TPU material: made of high-quality and scratch-resistant TPU material. Soft and lightweight, very comfortable to wear, leaves no air bubbles between the case and the screen, giving you an original viewing experience and touch experience. | Easy to install: no tools required. You don't need to remove the case, just align the holes with the watch buttons and put the case in place. Precise cutouts for quick access to screen, button and sensor. The case does not need to be removed when charging. | Fashion and Light: Soft and thin TPU materials make it easy to put on and take off your watch. Slim and lightweight, never strain your wrist from work to exercise. Give you a better user experience.</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>7</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>{'Compatible Devices': 'GM 165', 'Compatible Phone Models': 'Garmin Forerunner 165, Garmin Forerunner 165 Music', 'Special Features': 'Effective protective TPU material, full protection', 'Clarity': '10', 'Compatible Wearable Computer Models': 'Garmin Forerunner 165', 'Item Dimensions L x W': '10L x 6W centimetres', 'Unit Count': '2.0 unité', 'Number of Items': '2', 'Material': 'Silicone', 'Brand Name': 'TUTUO', 'Model Number': 'GM 165-HS+TM', 'Model Name': 'GM 165-HS+TM', 'Colour': 'Transparent/Green', 'Manufacturer': 'TUTUO', 'Part Number': 'GM 165-HS+TM', 'Best Sellers Rank': '4,130 in Electronics (See Top 100 in Electronics) 8 in Smartwatch Cases', 'ASIN': 'B0GHNJ6ZY3', 'Customer Reviews': '4.4  4.4 out of 5 stars   \n    (61)   \n\n\n 4.4 out of 5 stars'}</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Inconnu</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Aucune déclinaison</t>
+        </is>
+      </c>
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
@@ -5166,12 +7780,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>À collecter en Phase 2</t>
+          <t>Brand: Kamita</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>À collecter en Phase 2</t>
+          <t>Aucune description textuelle</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -5180,6 +7794,52 @@
         </is>
       </c>
       <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>[3 Pieces] Kamita Case Compatible with Garmin Vivoactive 5, Complete Protective Case with Tempered Glass Screen Protector, Shockproof Hard PC Bumper Case for Garmin Vivo Active 5 (Clear+Pink+White)</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>4.2 out of 5 stars</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>(192)</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>COMPATIBILITY: This specially designed Kamita protective case is compatible with Garmin Vivoactive 5, which can provide full protection for your watch. The screen protectors and protective case fit your watch perfectly. NOTE: This case does not fit other watch models. Please check the model of your watch before purchasing. | New material: This case compatible with Garmin Vivoactive 5 is made of hard and durable PC, which is more resistant to wear and does not lose its colors. The smooth surface ensures smooth gliding and tactile sensitivity, which gives you a better touch feeling. | Total protection: our Garmin Vivo Active 5 hard PC cases can cover all sides of your watch, ensuring total protection for your watch. Shockproof and scratch resistant design protects the watch from bumps and scratches. | Precise cutouts and easy installation: Our watch cover has a precise button cut-out that allows it to snap into place quickly and fit your watch precisely. Allows easy access to all buttons, sound holes, sensors and smartwatch functions. What's more, the snap-on design is easy to install and remove without any tools. It is also not necessary to remove the case to charge. | Package includes: The package includes 3 pieces of covers for Garmin Vivo Active 5. Humanized ergonomic house, air cushion technology to protect all areas. Suitable for men, women, girls, boys and any occasion.</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>7</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>{'Compatible Devices': 'Smartwatches', 'Form Factor': 'Case', 'Product Features': 'Shock and scratch resistant', 'Compatible Phone Models': 'Garmin Vivoactive 5', 'Water Resistance Level': 'Not Water Resistant', 'Colour': 'Transparent+Pink+White', 'Shell Type': 'Hard', 'Enclosure Material': 'Polycarbonate', 'Brand Name': 'Kamita', 'Unit Count': '3.0 count', 'Manufacturer': 'Kamita', 'Best Sellers Rank': '4,168 in Electronics (See Top 100 in Electronics) 9 in Smartwatch Cases', 'ASIN': 'B0DSZLRYTB', 'Customer Reviews': '4.2  4.2 out of 5 stars   \n    (192)   \n\n\n 4.2 out of 5 stars', 'Item Dimensions': '8 x 1 x 1.3 centimetres'}</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Inconnu</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Aucune déclinaison</t>
+        </is>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
@@ -5198,12 +7858,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>À collecter en Phase 2</t>
+          <t>Brand: Amizee</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>À collecter en Phase 2</t>
+          <t>Aucune description textuelle</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -5212,6 +7872,52 @@
         </is>
       </c>
       <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Amizee 2 in 1 Case Compatible with Apple Watch Series 11/10 46mm, Hard Metal Material Full Protection Rugged Anti-Scratch Case for iWatch 46mm, Black</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>4.1 out of 5 stars</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>(1,683)</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>【Compatible Models】Amizee cover only compatible with Apple Watch Series 11 (2025)/Series 10 46mm Cover. Note: Not suitable for other models and other types for smartwatch. Please confirm your watch size before placing an order. | 【Ultra 3/2/1 Second Change】Simple and tool-free installation transforms the appearance of your watch in seconds, allowing you to enjoy the Ultra 3/2/1 wearing experience, providing a stylish yet functional design and giving you a personal experience. The right button of the case has an updated built-in watch crown cover. (Note: crown does not work for ECG) | 【High quality metal casing】Made of high quality shockproof metal aluminum. Brighten up your Apple Watch and provide full protection without sacrificing beauty, and has long lasting protection against shocks. The snap-on design of the case is easy to install and remove. Charge directly, without removing the case. | 【Metal Bezel Protection】Raised edges around the screen for extra protection of the Apple Watch screen from scratches, bumps and accidental drops. Featuring an aluminum alloy frame, you will feel sturdy from the inside. (Note: does not include the built-in screen protector) | 【What you get】1 x black apple watch case 46 mm. If you have any defects or quality problems of our Apple Watch cases, please feel free to contact us, our customer service will reply you within 24 hours.</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>6</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>{'Compatible Devices': 'Apple Watch Series 10 46mm', 'Form Factor': 'Case', 'Compatible Device Size Maximum': '46 Millimetres', 'Product Features': 'Heavy Duty Protection', 'Compatible Phone Models': 'Apple Watch Series 11(2025)/Series 10 46mm', 'Water Resistance Level': 'Not Water Resistant', 'Colour': 'Black', 'Pattern': 'Sports', 'Theme': 'Sport', 'Shell Type': 'Hard', 'Enclosure Material': 'Aluminium', 'Brand Name': 'Amizee', 'Unit Count': '1.0 count', 'Manufacturer Part Number': 'BENQ3-CASE', 'Model Number': 'BENQ3-CASE', 'Manufacturer': 'Amizee', 'Age Range Description': 'Adult', 'Best Sellers Rank': '4,237 in Electronics (See Top 100 in Electronics) 10 in Smartwatch Cases', 'ASIN': 'B0DLKLY2RS', 'Customer Reviews': '4.1  4.1 out of 5 stars   \n    (1,683)   \n\n\n 4.1 out of 5 stars', 'Item Dimensions': '11 x 45 x 50 millimetres'}</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Inconnu</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Aucune déclinaison</t>
+        </is>
+      </c>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
@@ -5230,12 +7936,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>À collecter en Phase 2</t>
+          <t>Brand: Amizee</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>À collecter en Phase 2</t>
+          <t>Amizee 2 in 1 Metal Case Compatible with Samsung Galaxy Watch Ultra/Ultra 2 (2025) 47mm, Ultra Thin Hard PC Bumper Anti-Scratch Protective Case for Galaxy Watch 7/8 Ultra, Blue/White</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -5244,6 +7950,52 @@
         </is>
       </c>
       <c r="F12" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Amizee 2 in 1 Metal Case Compatible with Samsung Galaxy Watch Ultra/Ultra 2 (2025) 47mm, Ultra Thin Hard PC Bumper Anti-Scratch Protective Case for Galaxy Watch 7/8 Ultra, Blue/White</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>4.5 out of 5 stars</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>(907)</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Compatible models: Amizee cover only compatible with Samsung Galaxy Watch Ultra/Ultra 2 (2025) 47 mm. Note: Not suitable for other models and other types for smartwatch. Please confirm your watch size before placing an order. | 【High Quality Metal Casing】Made of high quality impact-resistant aluminum, metal and PC material. Brighten up your Samsung Galaxy Watch and ensure full protection without sacrificing beauty, and features long lasting protection against bumps. | 【Metal Bezel Protection】Raised edges around the screen provide extra protection for the Samsung Galaxy Watch screen from scratches, bumps and accidental drops. Featuring an aluminum alloy frame, you will feel sturdy from the inside. (Note: Does not include a built-in screen protector.) | 【Easy to snap on】 The snap-on design of the case is easy to install and remove. Simply press the side of the back cover case into the alignment of the crown hole. No tools, without removing the Galaxy Watch. Charge directly, without removing the case. Snap button design on the back prevents the watch from falling off. | 【What you get】1 x Blue/White Samsung Galaxy Watch Ultra/Ultra 2 (2025) 47 mm cover. If you have any defects or quality problems of our Apple Watch cases, please feel free to contact us, our customer service will reply you within 24 hours.</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>7</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>{'Compatible Devices': 'Samsung Galaxy Watch Ultra/Ultra 2 (2025) 47mm', 'Form Factor': 'Case', 'Compatible Device Size Maximum': '47 Millimetres', 'Product Features': 'Kickstand, Protection for demanding use, Wireless', 'Compatible Phone Models': 'Samsung Galaxy Watch Ultra/Ultra 2(2025) 47mm', 'Water Resistance Level': 'Not Water Resistant', 'Colour': 'Blue / white', 'Shell Type': 'Hard', 'Enclosure Material': 'Aluminium', 'Brand Name': 'Amizee', 'Manufacturer Part Number': 'GALAXYCASE-BK', 'Model Number': 'SGUltra-CASE-BUWhite', 'Manufacturer': 'Amizee', 'Best Sellers Rank': '4,485 in Electronics (See Top 100 in Electronics) 11 in Smartwatch Cases', 'ASIN': 'B0GCHZ4RP5', 'Customer Reviews': '4.5  4.5 out of 5 stars   \n    (907)   \n\n\n 4.5 out of 5 stars', 'Item Dimensions': '48 x 46 x 16 millimetres', 'Item Weight': '0.47 Ounces'}</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Inconnu</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Aucune déclinaison</t>
+        </is>
+      </c>
+      <c r="O12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
@@ -5262,12 +8014,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>À collecter en Phase 2</t>
+          <t>Visit the ivoler Store</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>À collecter en Phase 2</t>
+          <t>Fulfills Your Expectations Choose iVoler case, it does not make your watch look huge and bulky, but it is very thin and the case is matte, which makes your watch very elegant and gives it a natural look, so fashion and luxury. Perfect fit Precise hole cutouts make it easy to access all buttons. 360 Degree Full Protection Our case covers the full front and curved edges of the watch, provides full protection of your watch against dust, fingerprints, scratches, drop or dent to the ground. Sensitive Touch &amp; HD Clear 99% high transparency provides clear image quality and maintains the original touch sensitivity without affecting the use of touch. Easy to install and remove Ultra-soft material makes this case very flexible, easy to install and remove. This does not affect the use of load and strap after installation. After-sales Service We pay great attention to product quality problems and customer experienceIf you have any questions about our products, please feel free to contact us, we will reply you promptly within 24 hours. Note: These covers cannot support swimming as water will be trapped under the covers. During fitness or other sports, it may cause water mist between the watch screen and the screen protector. Please use a dry cloth to clean if water, sweat or moisture gets under the case, as it may affect the responsiveness to touch.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -5276,6 +8028,52 @@
         </is>
       </c>
       <c r="F13" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>ivoler 3 Pieces Case with Screen Protector for Huawei Watch GT 5 46mm, Full Protective Soft TPU Thin Shockproof Anti-Scratch Cover Case (2 Transparent + 1 Black)</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>4.3 out of 5 stars</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>(361)</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>[Applicable Model]---- Compatible with Huawei Watch GT 5 46mm (Not for Huawei Watch GT 5 41mm). This case is designed with precise cutouts for functional buttons, speaker hole, charging hole, etc.(The package only contains cases, watch and watch band are not included!) | [Full Protection] --- Our case covers the full front and curved edges of the watch, provides complete protection of your watch against dust, fingerprints, scratches, drops or bumps to the ground. | [Sensitive Touch and High Transparency]---- Made of premium TPU material, smooth, transparent and without influencing touch sensitivity. Gives you original touch sensitivity and high touch responsiveness. Hydrophobic and oleophobic screen coating can easily separate oil, fingerprints and other stains, make the screen easy to clean, prevent your watch screens from looking shabby and dull. | [Ultra Slim and Easy to Install] ---- Ultra thin and lightweight, never be a burden on your wrist from your work to your workout. Easy to wear and remove and designed to be compatible with the charger, you don't need to remove the protective case when charging. | [What you get] --- 3 x iVoler cases with built-in screen protector (2 transparent + 1 black). [Warm Tip]: Using this product in the gym or during sports activities may cause moisture (sweating) to build up between this product and the monitor screen. Use dry cloth to keep it dry if you have water, if you have any questions or product problems, please contact us, we will do the best service for you.</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>7</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>{'Compatible Devices': 'huawei watch gt 5 46mm', 'Item Hardness': '9H', 'Compatible Phone Models': 'huawei watch gt 5 46mm', 'Special Features': 'Rounded Edge, Shockproof', 'Screen Size': '46 Millimetres', 'Screen Surface Description': 'Glossy', 'Clarity': '99.9', 'Compatible Wearable Computer Models': 'Huawei WATCH GT, SUUNTO 5', 'Unit Count': '3.0 count', 'Number of Items': '3', 'Brand Name': 'ivoler', 'Model Name': 'iVoler Huawei Watch GT 5 46mm Screen Protector', 'Manufacturer': 'iVoler', 'Part Number': 'IVR-WATCHCASE4-00039', 'Best Sellers Rank': '3,967 in Electronics (See Top 100 in Electronics) 12 in Smartwatch Cases', 'ASIN': 'B0DJTDNSQN', 'Customer Reviews': '4.3  4.3 out of 5 stars   \n    (361)   \n\n\n 4.3 out of 5 stars', 'Material': 'Silicone'}</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Inconnu</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Aucune déclinaison</t>
+        </is>
+      </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
@@ -5294,12 +8092,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>À collecter en Phase 2</t>
+          <t>Brand: Amizee</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>À collecter en Phase 2</t>
+          <t>Aucune description textuelle</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -5308,6 +8106,52 @@
         </is>
       </c>
       <c r="F14" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Amizee 2 in 1 Case [2 Pieces] Compatible with Apple Watch SE 3/2/1 Series 6/5/4 40mm with Screen Protector, Full Coverage Anti-Scratch Case Cover for iWatch 40mm (Black)</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>4.1 out of 5 stars</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>(3,036)</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>【Compatible Models】Designed for Apple Watch SE 3/2/1 Series 6/5/4 40mm. NOTE: Not suitable for other models and other types of smartwatch. Please confirm your watch size before placing an order. | 【Full Body Protection】Made of high quality hard PC material, with built-in screen protector. 2 in 1 design provides robust 360 degree protection. Full body protection keeps your Apple Watch 40mm from scratches and drops. | High sensitivity touch: The high-transparency tempered glass screen protector provides original vision and touch experience; Ultra-thin, three-dimensional right-angle edge, the design is slimmer. | 【Precise Fit】Sensitive button covers allow responsive pressing; Easy access to Apple Watch button and functions with precise cutouts; Easy to install, charge directly, without removing the case. | 【WHAT YOU GET】2 x Black Apple Watch Case 40 mm; We offer a one-year warranty, please feel free to contact us for any problem, a satisfactory solution is promised forever.</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>6</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>{'Compatible Devices': 'Apple Watch Series 6/5/4/SE 40mm', 'Item Hardness': '9H', 'Compatible Phone Models': 'Apple Watch', 'Special Features': 'Robust protection, Scratch Resistant, Shockproof, screen protector', 'Finish Type': 'Glossy', 'Water Resistance Level': 'Waterproof', 'Screen Size': '44 Millimetres', 'Screen Surface Description': 'Matte', 'Clarity': '0.99', 'Compatible Wearable Computer Models': 'Apple Watch SE 40mm', 'Item Dimensions L x W': '43L x 38W millimetres', 'Unit Count': '1.0 unité', 'Number of Items': '2', 'Brand Name': 'Amizee', 'Model Number': 'APPLECASE-ZB', 'Model Name': 'CAZB-40-BLC', 'Colour': 'Black / Black', 'Manufacturer': 'Amizee', 'Part Number': 'CAZB-40-BLC', 'Item Weight': '0.18 Ounces', 'Included Components': 'Case for Apple Watch 40mm', 'Best Sellers Rank': '3,327 in Electronics (See Top 100 in Electronics) 13 in Smartwatch Cases 92 in Smartwatch Screen Protectors &amp; Foils', 'ASIN': 'B0C2CM7QWR', 'Customer Reviews': '4.1  4.1 out of 5 stars   \n    (3,036)   \n\n\n 4.1 out of 5 stars', 'Material': 'Polycarbonate, Tempered Glass'}</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Inconnu</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Aucune déclinaison</t>
+        </is>
+      </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
@@ -5326,12 +8170,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>À collecter en Phase 2</t>
+          <t>Brand: Bigqin</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>À collecter en Phase 2</t>
+          <t>Features: 【PC + High Quality Tempered Film】 The case does not affect touch sensitivity. Provide original touch sensitivity. 【Precise Cutouts】 Precise cutouts for all connections, speakers and buttons, easy access to all functions and controls. 【Full Protection】 The edge and screen protector are integrally formed. It protects the watch from scratches, collisions or other damage. Warm Tips: The screen protector case is not waterproof, please take it off while swimming or bathing. Moisture can be trapped in case you are exercising, please just use the microfiber cloth to wipe it off. Package contents: 4 x watch case with screen protector compatible with Xiaomi Redmi Watch 5 Active. Colour: Clear, Black, Blue, Pink</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -5340,6 +8184,52 @@
         </is>
       </c>
       <c r="F15" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>4-Piece Case Compatible with Xiaomi Redmi Watch 5 Active, Hard PC Case with Screen Protector, HD Case with Tempered Glass – Transparent, Black, Pink, Blue</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>4.2 out of 5 stars</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>(540)</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>1. Compatible models: Only compatible with Xiaomi Redmi Watch 5 Active, please confirm your watch model before purchasing. 4 colours per pack: transparent, black, pink, blue. | 2. Full protection: It protects the watch screen and sides from scratches, scrapes, chips, collisions or other damage. | 3. Material: durable PC case with screen protector. No influence on touch sensitivity, sensor functions work well with watch case. | 4. Easy to install: its snap-on design to avoid peeling off. Precise hole cutouts make it easy to access all buttons or buttons, slim and lightweight, no need to remove the watch case when charging. | 5. Tips: Recommended for removing the case when swimming or bathing. Moisture can be trapped in case when you exercise, please use the microfiber cloth to wipe it.</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>5</v>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>{'Compatible Devices': 'Smartwatch', 'Item Hardness': '9H', 'Compatible Phone Models': 'Xiaomi Redmi Watch 5 Active', 'Special Features': 'High quality tempered glass', 'Finish Type': 'Glossy', 'Water Resistance Level': 'Not Water Resistant', 'Screen Surface Description': 'Glossy', 'Clarity': '10', 'Unit Count': '4.0 count', 'Number of Items': '4', 'Material': 'Polycarbonate', 'Brand Name': 'Bigqin', 'Model Number': '13XMRMW5A-4PC', 'Model Name': 'Xiaomi Redmi Watch 5 Active Screen Protector 4-Pack', 'Customer Package Type': 'FFP Packaging', 'Colour': 'Redmi Watch 5 Active', 'Manufacturer': 'Bigqin', 'Part Number': 'B02', 'Included Components': 'Watch', 'Best Sellers Rank': '4,821 in Electronics (See Top 100 in Electronics) 14 in Smartwatch Cases', 'ASIN': 'B0DM4WJ7XH', 'Customer Reviews': '4.2  4.2 out of 5 stars   \n    (540)   \n\n\n 4.2 out of 5 stars'}</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Inconnu</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Aucune déclinaison</t>
+        </is>
+      </c>
+      <c r="O15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
@@ -5358,12 +8248,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>À collecter en Phase 2</t>
+          <t>Visit the ivoler Store</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>À collecter en Phase 2</t>
+          <t>Fulfills Your Expectations Choose iVoler case, it does not make your watch look huge and bulky, but it is very thin and the case is matte, which makes your watch very elegant and gives it a natural look, so fashion and luxury. Perfect fit Precise hole cutouts make it easy to access all buttons. 360 Degree Full Protection Our case covers the full front and curved edges of the watch, provides full protection of your watch against dust, fingerprints, scratches, drop or dent to the ground. Sensitive Touch &amp; HD Clear 99% high transparency provides clear image quality and maintains the original touch sensitivity without affecting the use of touch. Easy to install and remove Ultra-soft material makes this case very flexible, easy to install and remove. This does not affect the use of load and strap after installation. After-sales Service We pay great attention to product quality problems and customer experienceIf you have any questions about our products, please feel free to contact us, we will reply you promptly within 24 hours. Note: These covers cannot support swimming as water will be trapped under the covers. During fitness or other sports, it may cause water mist between the watch screen and the screen protector. Please use a dry cloth to clean if water, sweat or moisture gets under the case, as it may affect the responsiveness to touch.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -5372,6 +8262,52 @@
         </is>
       </c>
       <c r="F16" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>ivoler 3 Pieces Case with Screen Protector for Amazfit Active 2 (Round Edition), Full Protective Soft TPU Slim Shockproof Anti-Scratch Cover (2 Transparent + 1 Black)</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>4.3 out of 5 stars</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>(90)</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>[Applicable Model]---- Compatible with Amazfit Active 2 (Round Edition) (Not for Amazfit Active 2 Square Edition). This case is designed with precise cutouts for functional buttons, speaker hole, charging hole, etc.(The package only contains cases, watch and watch band are not included!) | [Full Protection] --- Our case covers the full front and curved edges of the watch, provides complete protection of your watch against dust, fingerprints, scratches, drops or bumps to the ground. | [Sensitive Touch and High Transparency]---- Made of premium TPU material, smooth, transparent and without influencing touch sensitivity. Gives you original touch sensitivity and high touch responsiveness. Hydrophobic and oleophobic screen coating can easily separate oil, fingerprints and other stains, make the screen easy to clean, prevent your watch screens from looking shabby and dull. | [Ultra Slim and Easy to Install] ---- Ultra thin and lightweight, never be a burden on your wrist from your work to your workout. Easy to wear and remove and designed to be compatible with the charger, you don't need to remove the protective case when charging. | [What you get] --- 3 x iVoler cases with built-in screen protector (2 transparent + 1 black). [Warm Tip]: Using this product in the gym or during sports activities may cause moisture (sweating) to build up between this product and the monitor screen. Use dry cloth to keep it dry if you have water, if you have any questions or product problems, please contact us, we will do the best service for you.</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>7</v>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>{'Compatible Devices': 'Smartwatch', 'Item Hardness': '9H', 'Compatible Phone Models': 'Amazfit Active 2 (Round Edition)', 'Special Features': 'Rounded Edge, Shockproof', 'Finish Type': 'Glossy', 'Screen Surface Description': 'Glossy', 'Clarity': '99.9', 'Item Dimensions L x W': '7.2L x 8.2W centimetres', 'Unit Count': '1.0 unité', 'Number of Items': '3', 'Material': 'Silicone', 'Brand Name': 'ivoler', 'Model Name': 'Amazfit Active 2 (Round Edition) Screen Protector', 'Colour': '2 Transparent + 1 Black', 'Manufacturer': 'iVoler', 'Part Number': 'IVR-WATCHCASE4-00073', 'Product Warranty': '1', 'Included Components': 'Case', 'Best Sellers Rank': '4,873 in Electronics (See Top 100 in Electronics) 15 in Smartwatch Cases', 'ASIN': 'B0DSW4V65Z', 'Customer Reviews': '4.3  4.3 out of 5 stars   \n    (90)   \n\n\n 4.3 out of 5 stars'}</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Inconnu</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Aucune déclinaison</t>
+        </is>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
@@ -5408,6 +8344,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5440,6 +8386,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5472,6 +8428,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5504,6 +8470,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5536,6 +8512,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5568,6 +8554,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5600,6 +8596,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5632,6 +8638,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5664,6 +8680,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -5696,6 +8722,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5728,6 +8764,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -5760,6 +8806,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -5792,6 +8848,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -5824,6 +8890,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5856,6 +8932,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -5888,6 +8974,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -5920,6 +9016,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -5952,6 +9058,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -5984,6 +9100,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -6016,6 +9142,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -6048,6 +9184,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -6080,6 +9226,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -6112,6 +9268,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -6144,6 +9310,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -6176,6 +9352,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -6208,6 +9394,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -6240,6 +9436,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -6272,6 +9478,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -6304,6 +9520,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -6336,6 +9562,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
+      <c r="P46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -6368,6 +9604,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -6400,6 +9646,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -6432,6 +9688,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
+      <c r="P49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -6464,6 +9730,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
+      <c r="P50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -6496,6 +9772,16 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr"/>
+      <c r="P51" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mise à jour des données et du nettoyage [Automatique]
</commit_message>
<xml_diff>
--- a/historique_bestsellers.xlsx
+++ b/historique_bestsellers.xlsx
@@ -9370,12 +9370,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Inconnu</t>
+          <t>Kamita</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Aucune description</t>
+          <t>A venir</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -9384,27 +9384,27 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H2" t="n">
         <v>1</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Aucune caractéristique</t>
+          <t>Plan B actif</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Non trouvé</t>
+          <t>Top Bestseller</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Aucune déclinaison</t>
+          <t>Aucune</t>
         </is>
       </c>
       <c r="L2" t="n">
@@ -9415,7 +9415,11 @@
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Données récupérées via Plan B</t>
+        </is>
+      </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
@@ -9434,12 +9438,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Inconnu</t>
+          <t>Visiter la boutique TOCOL</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Aucune description</t>
+          <t>A venir</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -9448,27 +9452,27 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H3" t="n">
         <v>1</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Aucune caractéristique</t>
+          <t>Plan B actif</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Non trouvé</t>
+          <t>Top Bestseller</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Aucune déclinaison</t>
+          <t>Aucune</t>
         </is>
       </c>
       <c r="L3" t="n">
@@ -9479,7 +9483,11 @@
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Données récupérées via Plan B</t>
+        </is>
+      </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
@@ -9498,12 +9506,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Inconnu</t>
+          <t>Amizee</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Aucune description</t>
+          <t>A venir</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -9512,27 +9520,27 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H4" t="n">
         <v>1</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Aucune caractéristique</t>
+          <t>Plan B actif</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Non trouvé</t>
+          <t>Top Bestseller</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Aucune déclinaison</t>
+          <t>Aucune</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -9543,7 +9551,11 @@
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Données récupérées via Plan B</t>
+        </is>
+      </c>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>

</xml_diff>